<commit_message>
Please communicate progress report changes and updates with me.
</commit_message>
<xml_diff>
--- a/Weekly_Reports/Week_of_April_23/ECE554_Progress_report.xlsx
+++ b/Weekly_Reports/Week_of_April_23/ECE554_Progress_report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Week</t>
   </si>
@@ -40,6 +40,10 @@
     <t>Petalinux image, display out</t>
   </si>
   <si>
+    <t xml:space="preserve">Awaiting PL tasks from Michael and for Josh M to finalize some Linux stuff
+</t>
+  </si>
+  <si>
     <t>Debug movement, colors</t>
   </si>
   <si>
@@ -49,6 +53,9 @@
     <t>Fixed pixel conversion &amp; input, AXI stream test image (WIP)</t>
   </si>
   <si>
+    <t>Redirected by PS changes.</t>
+  </si>
+  <si>
     <t>Finish game (30+ hours in one week; game is almost steam-ready). Starting poster, website and final report</t>
   </si>
   <si>
@@ -58,22 +65,28 @@
     <t>AXI Stream -&gt; DMA -&gt; Screen pipeline implemented</t>
   </si>
   <si>
+    <t>Redirected from poster, website, report tasks to audio</t>
+  </si>
+  <si>
+    <t>Last day for poster submission</t>
+  </si>
+  <si>
+    <t>Poster work, additional bug testing in game</t>
+  </si>
+  <si>
+    <t>Finish dispatch unit, render tiles</t>
+  </si>
+  <si>
+    <t>AXI4-S implementation</t>
+  </si>
+  <si>
+    <t>Completed audio as per agreed tasks</t>
+  </si>
+  <si>
     <t>Internal Demo</t>
   </si>
   <si>
-    <t>Last day for poster submission</t>
-  </si>
-  <si>
-    <t>Poster work, additional bug testing in game</t>
-  </si>
-  <si>
-    <t>Finish dispatch unit, render tiles</t>
-  </si>
-  <si>
-    <t>AXI4-S implementation</t>
-  </si>
-  <si>
-    <t>Started audio</t>
+    <t>Reworking audio per new requirements</t>
   </si>
   <si>
     <t>Last lab</t>
@@ -92,7 +105,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -103,6 +116,10 @@
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -119,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -128,6 +145,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -351,7 +374,7 @@
     <col customWidth="1" min="3" max="3" width="80.25"/>
     <col customWidth="1" min="4" max="4" width="40.13"/>
     <col customWidth="1" min="5" max="5" width="45.75"/>
-    <col customWidth="1" min="6" max="6" width="26.0"/>
+    <col customWidth="1" min="6" max="6" width="40.38"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -388,6 +411,9 @@
       <c r="E2" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="F2" s="3" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2">
@@ -395,56 +421,68 @@
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>12</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="2">
         <v>46128.0</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" ht="1.5" customHeight="1">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="2">
+        <v>46137.0</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="2">
         <v>46140.0</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>46137.0</v>
-      </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>19</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
       <c r="F6" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -452,7 +490,7 @@
         <v>46142.0</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -460,7 +498,7 @@
         <v>46143.0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -468,7 +506,7 @@
         <v>46145.0</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">

</xml_diff>